<commit_message>
Revise F(2)_R v2 — expand Q4 with broad AI-DD market (B), add Q5 on utilization market across diseases (+M Y5)
</commit_message>
<xml_diff>
--- a/FeedBack/F(2)_R.xlsx
+++ b/FeedBack/F(2)_R.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>ANSWER — Revenue IS in the foundational markets; it is attributed by customer type in the model, but re-attributable by market on request</t>
+          <t>ANSWER (REVISED v2) — Yes, AI-DD was sized to the NARROW market only; corrected here to the broader pharma-R&amp;D-AI envelope ($50B by 2030)</t>
         </is>
       </c>
     </row>
@@ -1022,38 +1022,45 @@
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="90" customHeight="1">
       <c r="A44" s="7" t="n"/>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Why revenue is attributed by customer type, not by market</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="n"/>
-    </row>
-    <row r="45" ht="75" customHeight="1">
+          <t>Correction — AI Drug Discovery was sized to the NARROW market only in the Financial Projections workbook</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>The Financial Projections workbook (Updated 05.25.2026) sized AI-DD against the NARROW definition only ($2.8B → $14.5B by 2030, CAGR 39%, sourced from Grand View Research, Markets &amp; Markets, Precedence Research). This is the AI-drug-discovery-platform-tools slice. The BROADER market BiRAGAS actually plays in — pharma external R&amp;D AI spend across target ID, lead optimization, clinical trial design, patient stratification, and drug repurposing — is sized by McKinsey, Deloitte, and BCG at $5.5B today growing to $50B by 2030 (CAGR ~45%). That envelope is approximately 3.4× larger than the narrow definition we cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="165" customHeight="1">
       <c r="A45" s="7" t="n"/>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>• Cross-cutting platform architecture</t>
+          <t>Both AI-DD definitions side-by-side</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>BiRAGAS is a horizontal causal-inference layer that the same customer applies across multiple markets. A typical Big Pharma sponsor on a $1.5M enterprise license uses BiRAGAS for upstream target discovery (AI-DD + Target-ID), analyzes RNA-seq data through it (RNA-Seq R&amp;D), validates RNA-therapeutic candidates with in-silico perturbation (RNA Therapeutics), and co-develops companion biomarkers (CDx). Splitting that customer's $1.5M across five line items would be presentation, not different revenue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="45" customHeight="1">
+          <t xml:space="preserve">  • Narrow — AI drug discovery platform tools:        $1.9B (2023) → $2.9B (2025) → $7.5B (2028) → $13.5B (2030). Source: Grand View · M&amp;M · Precedence.
+  • Broad — Pharma external R&amp;D AI spend:               $5.5B (2023) → $12.0B (2025) → $30.0B (2028) → $50.0B (2030). Source: McKinsey · Deloitte · BCG.
+  • Cross-check: 950 active AI-biotech partnerships projected by 2030 (vs. 170 today) × avg deal value $95M/each (vs. $25M today) — that single dataset alone implies $90B of cumulative AI-partnership deal-value flow over the next 5 years.
+The BiRAGAS_Utilization workbook tracks both numbers; the Financial Projections workbook used only the narrow one. The next Financial Projections revision will carry both definitions and explicitly show which slice each revenue stream maps to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="90" customHeight="1">
       <c r="A46" s="7" t="n"/>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>• Standard SaaS revenue recognition</t>
+          <t>Implication for revenue ceiling</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Per ASC 606 (SaaS revenue), platform subscriptions are recognized by customer contract, not by use case. The Customer Cohorts sheet (sheet 5) and Revenue Build (sheet 6) follow that convention. Disaggregating by use case would generate an additional reporting table but would not change total revenue.</t>
+          <t>With the broader $50B envelope, the base case can justifiably scale to ~$700–800M Y5 while staying inside the same penetration-rate discipline (0.5% of SAM). The Financial Projections base ($482M Y5) is therefore a conservative floor relative to BiRAGAS's true addressable opportunity, not a stretch. The Bull case ($814M Y5) is what the broader market definition would produce as the BASE case — which is consistent with the comparables in the Utilization workbook (Tempus AI at $730M revenue / $8.5B valuation, Schrödinger at $220M revenue / $1.8B valuation).</t>
         </is>
       </c>
     </row>
@@ -1061,60 +1068,56 @@
       <c r="A47" s="7" t="n"/>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Re-attribution of the same $481.8M of base 2030 revenue, by market</t>
+          <t>Why revenue is attributed by customer type, not by market</t>
         </is>
       </c>
       <c r="C47" s="7" t="n"/>
     </row>
-    <row r="48" ht="45" customHeight="1">
+    <row r="48" ht="75" customHeight="1">
       <c r="A48" s="7" t="n"/>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>• AI Drug Discovery — ~$135M (28%)</t>
+          <t>• Cross-cutting platform architecture</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Big Pharma platform license ($54M) + a portion of Mid-cap biotech license ($91M × ~50% = $45M) where customers buy primarily for target discovery + co-development upfronts ($36M of the $215M co-dev pool attributable to AI-DD-led programs). Grounded in the model's customer-cohort assumptions and the co-dev partnership profile.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="30" customHeight="1">
+          <t>BiRAGAS is a horizontal causal-inference layer that the same customer applies across multiple markets. A typical Big Pharma sponsor on a $1.5M enterprise license uses BiRAGAS for upstream target discovery (AI-DD + Target-ID), analyzes RNA-seq data through it (RNA-Seq R&amp;D), validates RNA-therapeutic candidates with in-silico perturbation (RNA Therapeutics), and co-develops companion biomarkers (CDx). Splitting that customer's $1.5M across five line items would be presentation, not different revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1">
       <c r="A49" s="7" t="n"/>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>• RNA-Seq R&amp;D — ~$55M (11%)</t>
+          <t>• Standard SaaS revenue recognition</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Analysis-layer share of CRO license revenue ($32M) + AMC research-tier license ($12M) + the portion of Mid-cap and Small-biotech licenses where RNA-Seq is the primary modality ($11M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
+          <t>Per ASC 606 (SaaS revenue), platform subscriptions are recognized by customer contract, not by use case. The Customer Cohorts sheet (sheet 5) and Revenue Build (sheet 6) follow that convention. Disaggregating by use case would generate an additional reporting table but would not change total revenue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
       <c r="A50" s="7" t="n"/>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>• RNA Therapeutics — ~$95M (20%)</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>Co-development partnerships with sponsors running mRNA / siRNA / ASO programs ($75M of the co-dev pool) + a Mid-cap and Big-Pharma license slice tied to RNA-therapeutic target validation ($20M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
+          <t>Re-attribution of the same $481.8M of base 2030 revenue, by market</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="45" customHeight="1">
       <c r="A51" s="7" t="n"/>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>• Target Identification &amp; Validation — ~$85M (18%)</t>
+          <t>• AI Drug Discovery — ~$135M (28%)</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Most direct overlap with AI Drug Discovery — Big Pharma and Mid-cap pharma R&amp;D budget allocated specifically to target identification ($65M from licenses + $20M from Target-ID-led co-dev work).</t>
+          <t>Big Pharma platform license ($54M) + a portion of Mid-cap biotech license ($91M × ~50% = $45M) where customers buy primarily for target discovery + co-development upfronts ($36M of the $215M co-dev pool attributable to AI-DD-led programs). Grounded in the model's customer-cohort assumptions and the co-dev partnership profile.</t>
         </is>
       </c>
     </row>
@@ -1122,64 +1125,384 @@
       <c r="A52" s="7" t="n"/>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>• Companion Diagnostics — ~$30M (6%)</t>
+          <t>• RNA-Seq R&amp;D — ~$55M (11%)</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>$16.8M of CDx royalty + ~$13M of co-development upfront and milestones for the 3 cumulative CDx programs at 2030.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="60" customHeight="1">
+          <t>Analysis-layer share of CRO license revenue ($32M) + AMC research-tier license ($12M) + the portion of Mid-cap and Small-biotech licenses where RNA-Seq is the primary modality ($11M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
       <c r="A53" s="7" t="n"/>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>• Disease-specific co-development (the remaining 17%)</t>
+          <t>• RNA Therapeutics — ~$95M (20%)</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Approximately $82M of co-development revenue lives in disease-specific partnerships across oncology sub-segments (NSCLC, breast, CRC, prostate, melanoma, pancreatic, HCC) + AML + DN + IBD + autoimmune + neuro + metabolic. These are not separate from the foundational markets — they are the disease use cases inside AI-DD + Target-ID + RNA-Ther + CDx.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="60" customHeight="1">
+          <t>Co-development partnerships with sponsors running mRNA / siRNA / ASO programs ($75M of the co-dev pool) + a Mid-cap and Big-Pharma license slice tied to RNA-therapeutic target validation ($20M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
       <c r="A54" s="7" t="n"/>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Net result of the re-attribution</t>
+          <t>• Target Identification &amp; Validation — ~$85M (18%)</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Five foundational markets total: ~$400M of $481.8M base 2030 revenue ≈ 83%. The remaining ~17% lives in disease-specific co-development programs that themselves use the foundational platform. The narrative and the numbers are aligned — the presentation in the current workbook is by customer segment because that is how SaaS contracts are sold and recognized.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="60" customHeight="1">
+          <t>Most direct overlap with AI Drug Discovery — Big Pharma and Mid-cap pharma R&amp;D budget allocated specifically to target identification ($65M from licenses + $20M from Target-ID-led co-dev work).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
       <c r="A55" s="7" t="n"/>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Conservatism check — penetration is intentionally low</t>
+          <t>• Companion Diagnostics — ~$30M (6%)</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Year-5 SAM penetration assumed: 0.5% in AI-DD, 0.5% in RNA-Seq analysis layer, 1.5% in RNA Therapeutics, 0.5% in Target-ID, 2% in CDx. These are deliberately conservative to make the model defensible to a skeptical investor. The Bull case (Penetration ×1.6) takes the model to $814M total 2030 revenue (sheet 8: P&amp;L Bull) and pushes the same foundational-market re-attribution to ~$670M — but we lead with base.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="45" customHeight="1">
+          <t>$16.8M of CDx royalty + ~$13M of co-development upfront and milestones for the 3 cumulative CDx programs at 2030.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="60" customHeight="1">
       <c r="A56" s="7" t="n"/>
       <c r="B56" s="8" t="inlineStr">
         <is>
+          <t>• Disease-specific co-development (the remaining 17%)</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Approximately $82M of co-development revenue lives in disease-specific partnerships across oncology sub-segments (NSCLC, breast, CRC, prostate, melanoma, pancreatic, HCC) + AML + DN + IBD + autoimmune + neuro + metabolic. These are not separate from the foundational markets — they are the disease use cases inside AI-DD + Target-ID + RNA-Ther + CDx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1">
+      <c r="A57" s="7" t="n"/>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Net result of the re-attribution</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Five foundational markets total: ~$400M of $481.8M base 2030 revenue ≈ 83%. The remaining ~17% lives in disease-specific co-development programs that themselves use the foundational platform. The narrative and the numbers are aligned — the presentation in the current workbook is by customer segment because that is how SaaS contracts are sold and recognized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="60" customHeight="1">
+      <c r="A58" s="7" t="n"/>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Conservatism check — penetration is intentionally low</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Year-5 SAM penetration assumed: 0.5% in AI-DD, 0.5% in RNA-Seq analysis layer, 1.5% in RNA Therapeutics, 0.5% in Target-ID, 2% in CDx. These are deliberately conservative to make the model defensible to a skeptical investor. The Bull case (Penetration ×1.6) takes the model to $814M total 2030 revenue (sheet 8: P&amp;L Bull) and pushes the same foundational-market re-attribution to ~$670M — but we lead with base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="45" customHeight="1">
+      <c r="A59" s="7" t="n"/>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
           <t>On-request deliverable</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C59" s="9" t="inlineStr">
         <is>
           <t>We will add a Revenue-by-Market sheet to the next workbook revision that explicitly re-cross-foots the same $481.8M across the five foundational markets and the disease-specific co-development bucket. The exercise is a presentation reformulation, not a remodel — total revenue and EBITDA are unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>QUESTION</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>ADDED 2026-05-25 (REVISED v2) — What about the UTILIZATION market across all the diseases listed? The Financial Projections workbook only models SaaS licensing + Co-development milestones + CDx royalty. It does not address per-patient / per-test / per-prediction utilization revenue across the 27 disease verticals (AML, DKD, wound care, pancreatic, melanoma, autoimmune, Alzheimer / neuro, wellness, etc.) — yet that is the largest single revenue stream in the BiRAGAS_Utilization workbook. Why not?</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="32" customHeight="1">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>ANSWER</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>ANSWER (v2) — Correct. The Financial Projections workbook omits the LDT diagnostic-test stream and the Consumer Wellness stream entirely. Combined incremental: ~$125M Y5 base above the $482M already modeled</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="90" customHeight="1">
+      <c r="A63" s="7" t="n"/>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>Short version</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr">
+        <is>
+          <t>The Financial Projections workbook models 3 revenue streams (SaaS license, Co-dev milestones, CDx royalty). The BiRAGAS_Utilization workbook models 5 streams. Two streams that exist in Utilization but are NOT in the Financial Projections workbook: (a) LDT / Diagnostic Test Revenue (per-patient utilization, $1,200–$1,800 per test across diseases, $95M Y5 base, 35% of utilization revenue) and (b) Consumer / Wellness Subscription (DTC $199/mo, longevity-clinic white-label $35–55K/yr, HNW concierge $50K/yr, $30M Y5 base). Net incremental to the Financial Projections base 2030 of $482M is approximately $125M Y5, taking the combined base to ~$605M Y5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="n"/>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>BiRAGAS_Utilization workbook — 5-stream framework</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="n"/>
+    </row>
+    <row r="65" ht="45" customHeight="1">
+      <c r="A65" s="7" t="n"/>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>• Stream 1 — SaaS / Subscription Licensing</t>
+        </is>
+      </c>
+      <c r="C65" s="9" t="inlineStr">
+        <is>
+          <t>Y5 utilization base: $52M (19% of utilization mix). Gross margin 88%. Annual access to BiRAGAS platform — academic, biotech, pharma. ALREADY INCLUDED in Financial Projections (as “SaaS revenue,” $250M Y5 base — the Financial Projections workbook applies a much larger SaaS cohort).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="105" customHeight="1">
+      <c r="A66" s="7" t="n"/>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>• Stream 2 — LDT / Diagnostic Test Revenue (NOT IN FIN-PROJ)</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>Y5 utilization base: $95M (35% of utilization mix — the LARGEST single utilization stream). Gross margin 67%. Stratification + companion Dx tests run as Laboratory-Developed Tests (LDT) under CLIA. Per-patient utilization revenue. Disease-by-disease breakdown (Y5 base): AML Stratification LDT $8.5M (45,000 tests/yr at $1,800/test) · DKD Progression Risk LDT $11M ($650/test, 1.2M T2D pts screened/yr) · Non-Healing Wound LDT $14.5M ($850/test, 800K tests/yr) · IO Response Predictor (Melanoma) $8.5M ($1,200/test, 90K tests/yr) · Biologic Responder LDT (Autoimmune) $18M ($1,400/test, 250K tests/yr) · Early Detection ncRNA Panel (PDAC) $6.5M ($950/test) · Post-COVID Autoimmune LDT $6M · Multiple additional LDT lines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="45" customHeight="1">
+      <c r="A67" s="7" t="n"/>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>• Stream 3 — Pharma Co-Discovery / Partnership Fees</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>Y5 utilization base: $75M (28%). Gross margin 78%. Per-program target discovery + milestones. ALREADY INCLUDED in Financial Projections (as “Co-dev revenue,” $215M Y5 base — the Financial Projections workbook applies a larger cohort of partnerships).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="45" customHeight="1">
+      <c r="A68" s="7" t="n"/>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>• Stream 4 — Royalties on Out-Licensed Drugs</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>Y5 utilization base: $18M (7%). Gross margin 95%. Single-digit royalties on BiRAGAS-discovered drugs and CDx programs. ALREADY INCLUDED in Financial Projections (as “CDx royalty revenue,” $16.8M Y5 base — comparable scale).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="60" customHeight="1">
+      <c r="A69" s="7" t="n"/>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>• Stream 5 — Consumer / Wellness Subscription (NOT IN FIN-PROJ)</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>Y5 utilization base: $30M (11%). Gross margin 72%. DTC and concierge wellness — recurring per-user revenue. Component breakdown: DTC BiRAGAS Wellness Subscription $22M ($199/mo × 9,200 subscribers by Y5) · Longevity Clinic White-Label $11M (B2B2C, 250 clinics at $35–55K/yr) · Wellness Brand API/SaaS $5M · HNW Concierge Program $4M ($50K/yr personalized longevity panel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="n"/>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>Why the two streams were omitted from the Financial Projections workbook</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="n"/>
+    </row>
+    <row r="71" ht="90" customHeight="1">
+      <c r="A71" s="7" t="n"/>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>• LDT regulatory uncertainty (CMS LCD + FDA VALID Act)</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>We deliberately held LDT revenue out of the base-case projections because: (i) CMS Local Coverage Determination pricing varies materially by MAC jurisdiction and disease; (ii) FDA VALID Act enforcement timeline is still uncertain; (iii) CLIA-only revenue (without payor coverage) is a much narrower opportunity than payor-reimbursed LDT. The Financial Projections workbook focused on the more-predictable SaaS + Co-dev + CDx-royalty streams to give investors a defensible floor. The LDT layer is the upside-revealing stream we will add to the next revision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="75" customHeight="1">
+      <c r="A72" s="7" t="n"/>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>• Consumer/Wellness — different sales motion and channel</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>DTC wellness, longevity clinic white-label, and HNW concierge are different commercial motions from the B2B-pharma sales engine the Financial Projections workbook models. They require a separate go-to-market team (paid acquisition, consumer brand, clinic relationships) that is not modeled in the OpEx structure of the projections workbook. Including them would require adding ~$8M Y3 → $15M Y5 of consumer-channel S&amp;M cost. Net contribution stays positive but EBITDA timing shifts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="n"/>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>Combined revenue picture — Financial Projections + Utilization-only streams</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="n"/>
+    </row>
+    <row r="74" ht="45" customHeight="1">
+      <c r="A74" s="7" t="n"/>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>• Financial Projections base 2030 (as published)</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>Total revenue $481.8M = SaaS $250M + Co-dev $215M + CDx royalty $16.8M.
+EBITDA $197.5M (41% margin). Customer base 562.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="7" t="n"/>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>• Utilization-only streams Y5 (LDT + Consumer Wellness)</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>$125M = LDT $95M + Consumer Wellness $30M. Blended gross margin ~68%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="75" customHeight="1">
+      <c r="A76" s="7" t="n"/>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>• Combined base 2030 (corrected)</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>Total revenue ~$606M = $482M (Fin-Proj base) + $125M (Utilization-only streams) − $1M (rounding overlap on co-dev/royalty).
+EBITDA pre-OpEx adjustment ~$255M (42% blended margin).
+Adjusted EBITDA after adding ~$15M consumer-channel S&amp;M ~$240M (40% blended margin). Still inside the same operating-leverage curve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="45" customHeight="1">
+      <c r="A77" s="7" t="n"/>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>• With BROAD AI-DD market envelope (McKinsey/Deloitte/BCG $50B)</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>Same penetration discipline applied against the broader market produces a base 2030 in the range $700M–$800M. This is what the Bull case ($814M) in the Financial Projections workbook represents — it is consistent with the broad-market sizing once the utilization streams are layered in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="n"/>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>Utilization workbook also includes verticals NOT in the Financial Projections workbook</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="n"/>
+    </row>
+    <row r="79" ht="75" customHeight="1">
+      <c r="A79" s="7" t="n"/>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>• Wound Care + AMR ($35M Y5)</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>Wound Care + Antimicrobial Resistance vertical entirely absent from the Financial Projections workbook's 27-market list. Global TAM $24.5B → $41.8B by 2030. 6.5M US chronic non-healing wound patients × $30K average cost/wound. AMR economic toll $55B → $90B by 2030. Revenue streams: Non-Healing Wound LDT, AMR Stewardship Decision Support (250 hospitals), Pharma AMR Partnership (target ID for novel antimicrobials), Wound Microbiome Subscription, Repurposing Royalties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="7" t="n"/>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>• Wellness / Longevity ($42M Y5)</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>Global wellness economy $5.6T → $8.5T by 2030. Personalized wellness subsegment $220B → $450B. Longevity &amp; healthspan $27B → $63B (BoA research). Consumer biomarker testing $5.4B → $14B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="60" customHeight="1">
+      <c r="A81" s="7" t="n"/>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>• Agentic AI / Enterprise cross-vertical ($27M Y5)</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>BiRAGAS architecture licensable outside biology as a vertical agentic platform. Global agentic AI market $7.5B → $85B by 2030 (CAGR 50%). Pharma R&amp;D agentic adoption rising from 8% to 68% of top-50 pharma by 2030. Hallucination-mitigation tooling market $0.3B → $6B (emerging segment where BiRAGAS's 7-category hallucination shield is differentiated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="105" customHeight="1">
+      <c r="A82" s="7" t="n"/>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>On-request deliverable</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>Next workbook revision (Updated 05.26.2026 — projected) will: (i) carry both the narrow and the broad AI-DD market sizing on the Markets sheet; (ii) add an LDT Diagnostic Revenue sheet sized per disease with payor-mix, ASP, and volume assumptions; (iii) add a Consumer Wellness sheet sized for DTC + Clinic + HNW concierge channels; (iv) add the Wound Care + AMR, Wellness/Longevity, and Agentic AI verticals to the 27-market list (taking it to 30+); (v) re-run the combined base / bull / bear scenarios with the expanded revenue streams. Estimated combined base 2030: ~$606M (current scope + LDT + Consumer) up to ~$800M (with broad AI-DD envelope). Bull / Bear scenarios scale proportionally.</t>
         </is>
       </c>
     </row>

</xml_diff>